<commit_message>
Updating website tick boxes and legend
</commit_message>
<xml_diff>
--- a/mapping/r/website_map/Website map - sites.xlsx
+++ b/mapping/r/website_map/Website map - sites.xlsx
@@ -13,11 +13,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={020ad635-70ff-4dd6-a148-5a1130336ba0}</author>
-    <author>tc={695dd486-ac34-40ad-868c-632e3ab38081}</author>
+    <author>tc={1a854dcb-9ccf-42b8-993e-950ea7561269}</author>
+    <author>tc={d93c322d-3737-4d3c-8eda-96e09e1e9f58}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{020ad635-70ff-4dd6-a148-5a1130336ba0}" ref="G11">
+    <comment authorId="0" xr:uid="{1a854dcb-9ccf-42b8-993e-950ea7561269}" ref="G11">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -26,7 +26,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{695dd486-ac34-40ad-868c-632e3ab38081}" ref="G10">
+    <comment authorId="1" xr:uid="{d93c322d-3737-4d3c-8eda-96e09e1e9f58}" ref="G10">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="56">
   <si>
     <t>name</t>
   </si>
@@ -63,7 +63,7 @@
     <t>future photo</t>
   </si>
   <si>
-    <t>Ten Pound Bay</t>
+    <t>Ten Pound Bay Nursery</t>
   </si>
   <si>
     <t>coral nursery</t>
@@ -72,58 +72,64 @@
     <t>nursery_tpb.jpg</t>
   </si>
   <si>
-    <t>York Island</t>
+    <t>York Island Nursery</t>
   </si>
   <si>
     <t>nursery_york.jpg</t>
   </si>
   <si>
-    <t>Jumby Bay</t>
+    <t>Jumby Bay Nursery</t>
   </si>
   <si>
     <t>nursery_jumby.jpg</t>
   </si>
   <si>
-    <t>Cades Reef Sculpture Garden</t>
+    <t>Cades Sculpture Nursery</t>
   </si>
   <si>
     <t>nursery_cadessculptures.jpg</t>
   </si>
   <si>
-    <t>coral restoration site</t>
+    <t>Ten Pound Bay Restoration Site</t>
+  </si>
+  <si>
+    <t>coral restoration</t>
   </si>
   <si>
     <t>restoration_tpb.jpg</t>
   </si>
   <si>
-    <t>Spithead Reef</t>
+    <t>Spithead Reef Restoration Site</t>
   </si>
   <si>
     <t>restoration_spithead.jpg</t>
   </si>
   <si>
-    <t>Cades Reef Outer Reef</t>
+    <t>Cades Outer Restoration Site</t>
   </si>
   <si>
     <t>restoration_cadesouter.jpg</t>
   </si>
   <si>
-    <t>Cades Reef Inner</t>
+    <t>Cades Inner Restoration Site</t>
   </si>
   <si>
     <t>restoration_cadesinner.jpg</t>
   </si>
   <si>
+    <t>Cades Sculpture Restoration Site</t>
+  </si>
+  <si>
     <t>restoration_cadessculptures.jpg</t>
   </si>
   <si>
-    <t>South Bird Island</t>
+    <t>South Bird Island Restoration Site</t>
   </si>
   <si>
     <t>restoration_southbird.jpg</t>
   </si>
   <si>
-    <t>Hydrophone</t>
+    <t>Marine Mammal Monitoring Hydrophone</t>
   </si>
   <si>
     <t>marine mammal monitoring</t>
@@ -755,7 +761,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Molly Wilson" id="{6f470ca4-a187-4a62-8a4a-f04a584d2a02}" providerId="google-sheets"/>
+  <x18tc:person displayName="Molly Wilson" id="{f4feec1c-5f76-482d-9e09-3993e4891d39}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -955,10 +961,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="G11" dT="2026-04-02T20:23:42.00" personId="{6f470ca4-a187-4a62-8a4a-f04a584d2a02}" id="{020ad635-70ff-4dd6-a148-5a1130336ba0}" done="0">
+  <x18tc:threadedComment ref="G11" dT="2026-04-02T20:23:42.00" personId="{f4feec1c-5f76-482d-9e09-3993e4891d39}" id="{1a854dcb-9ccf-42b8-993e-950ea7561269}" done="0">
     <x18tc:text xml:space="preserve">pending</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="G10" dT="2026-04-02T20:23:36.00" personId="{6f470ca4-a187-4a62-8a4a-f04a584d2a02}" id="{695dd486-ac34-40ad-868c-632e3ab38081}" done="0">
+  <x18tc:threadedComment ref="G10" dT="2026-04-02T20:23:36.00" personId="{f4feec1c-5f76-482d-9e09-3993e4891d39}" id="{d93c322d-3737-4d3c-8eda-96e09e1e9f58}" done="0">
     <x18tc:text xml:space="preserve">pending</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1080,10 +1086,10 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C6" s="7">
         <v>17.067505</v>
@@ -1094,9 +1100,8 @@
       <c r="E6" s="9">
         <v>44713.0</v>
       </c>
-      <c r="F6" s="10"/>
-      <c r="G6" s="6" t="s">
-        <v>17</v>
+      <c r="F6" s="6" t="s">
+        <v>18</v>
       </c>
       <c r="H6" s="10"/>
       <c r="I6" s="10"/>
@@ -1119,10 +1124,10 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="C7" s="2">
         <v>17.092666</v>
@@ -1134,15 +1139,15 @@
         <v>45748.0</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>16</v>
+        <v>21</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="C8" s="2">
         <v>17.006126</v>
@@ -1154,15 +1159,15 @@
         <v>45658.0</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="C9" s="2">
         <v>17.014637</v>
@@ -1174,15 +1179,15 @@
         <v>45566.0</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C10" s="8">
         <v>17.008369</v>
@@ -1193,9 +1198,8 @@
       <c r="E10" s="9">
         <v>46082.0</v>
       </c>
-      <c r="F10" s="10"/>
       <c r="G10" s="6" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H10" s="10"/>
       <c r="I10" s="10"/>
@@ -1218,10 +1222,10 @@
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C11" s="8">
         <v>17.143356</v>
@@ -1234,7 +1238,7 @@
       </c>
       <c r="F11" s="10"/>
       <c r="G11" s="6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H11" s="10"/>
       <c r="I11" s="10"/>
@@ -1257,10 +1261,10 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C12" s="11">
         <v>16.991873</v>
@@ -1272,15 +1276,15 @@
         <v>45627.0</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C13" s="11">
         <v>17.104355</v>
@@ -1294,10 +1298,10 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C14" s="13">
         <v>17.098221</v>
@@ -1312,10 +1316,10 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C15" s="17">
         <v>17.126645</v>
@@ -1330,10 +1334,10 @@
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" s="18">
         <v>16.9975333333</v>
@@ -1348,10 +1352,10 @@
     </row>
     <row r="17">
       <c r="A17" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C17" s="18">
         <v>16.9975333333</v>
@@ -1366,10 +1370,10 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C18" s="18">
         <v>16.9975333333</v>
@@ -1384,10 +1388,10 @@
     </row>
     <row r="19">
       <c r="A19" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C19" s="11">
         <v>17.055765</v>
@@ -1402,10 +1406,10 @@
     </row>
     <row r="20">
       <c r="A20" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C20" s="18">
         <v>16.9975333333</v>
@@ -1420,10 +1424,10 @@
     </row>
     <row r="21">
       <c r="A21" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C21" s="18">
         <v>16.9975333333</v>
@@ -1438,10 +1442,10 @@
     </row>
     <row r="22">
       <c r="A22" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C22" s="18">
         <v>17.57545</v>
@@ -1456,10 +1460,10 @@
     </row>
     <row r="23">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C23" s="18">
         <v>16.9975333333</v>
@@ -1474,10 +1478,10 @@
     </row>
     <row r="24">
       <c r="A24" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C24" s="21">
         <v>17.1641666667</v>
@@ -1492,10 +1496,10 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C25" s="18">
         <v>17.03195</v>
@@ -1510,10 +1514,10 @@
     </row>
     <row r="26">
       <c r="A26" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C26" s="18">
         <v>17.03526</v>
@@ -1528,10 +1532,10 @@
     </row>
     <row r="27">
       <c r="A27" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C27" s="18">
         <v>17.03296</v>
@@ -1546,10 +1550,10 @@
     </row>
     <row r="28">
       <c r="A28" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C28" s="18">
         <v>17.03535</v>
@@ -1564,10 +1568,10 @@
     </row>
     <row r="29">
       <c r="A29" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C29" s="18">
         <v>17.03425</v>
@@ -1582,10 +1586,10 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C30" s="18">
         <v>17.03425</v>
@@ -1600,10 +1604,10 @@
     </row>
     <row r="31">
       <c r="A31" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C31" s="18">
         <v>17.03425</v>
@@ -1618,10 +1622,10 @@
     </row>
     <row r="32">
       <c r="A32" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C32" s="18">
         <v>17.03326</v>
@@ -1636,10 +1640,10 @@
     </row>
     <row r="33">
       <c r="A33" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C33" s="18">
         <v>17.03358</v>
@@ -1654,10 +1658,10 @@
     </row>
     <row r="34">
       <c r="A34" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C34" s="18">
         <v>17.05387</v>

</xml_diff>

<commit_message>
Finished website map app!
</commit_message>
<xml_diff>
--- a/mapping/r/website_map/Website map - sites.xlsx
+++ b/mapping/r/website_map/Website map - sites.xlsx
@@ -13,11 +13,11 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={1a854dcb-9ccf-42b8-993e-950ea7561269}</author>
-    <author>tc={d93c322d-3737-4d3c-8eda-96e09e1e9f58}</author>
+    <author>tc={8ae9ac8e-0cbb-4117-bd88-108af5d8e146}</author>
+    <author>tc={8c53f43b-1065-4a92-90f5-08e778ce36b0}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{1a854dcb-9ccf-42b8-993e-950ea7561269}" ref="G11">
+    <comment authorId="0" xr:uid="{8ae9ac8e-0cbb-4117-bd88-108af5d8e146}" ref="G10">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -26,7 +26,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{d93c322d-3737-4d3c-8eda-96e09e1e9f58}" ref="G10">
+    <comment authorId="1" xr:uid="{8c53f43b-1065-4a92-90f5-08e778ce36b0}" ref="G11">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -694,11 +694,11 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
@@ -761,7 +761,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Molly Wilson" id="{f4feec1c-5f76-482d-9e09-3993e4891d39}" providerId="google-sheets"/>
+  <x18tc:person displayName="Molly Wilson" id="{476a260c-d452-4c9d-acab-8a75b4c1d0a5}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -961,10 +961,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="G11" dT="2026-04-02T20:23:42.00" personId="{f4feec1c-5f76-482d-9e09-3993e4891d39}" id="{1a854dcb-9ccf-42b8-993e-950ea7561269}" done="0">
+  <x18tc:threadedComment ref="G11" dT="2026-04-02T20:23:42.00" personId="{476a260c-d452-4c9d-acab-8a75b4c1d0a5}" id="{8c53f43b-1065-4a92-90f5-08e778ce36b0}" done="0">
     <x18tc:text xml:space="preserve">pending</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="G10" dT="2026-04-02T20:23:36.00" personId="{f4feec1c-5f76-482d-9e09-3993e4891d39}" id="{d93c322d-3737-4d3c-8eda-96e09e1e9f58}" done="0">
+  <x18tc:threadedComment ref="G10" dT="2026-04-02T20:23:36.00" personId="{476a260c-d452-4c9d-acab-8a75b4c1d0a5}" id="{8ae9ac8e-0cbb-4117-bd88-108af5d8e146}" done="1">
     <x18tc:text xml:space="preserve">pending</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -1085,48 +1085,30 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="6">
         <v>17.067505</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="3">
         <v>-61.66417</v>
       </c>
-      <c r="E6" s="9">
+      <c r="E6" s="5">
         <v>44713.0</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="10"/>
-      <c r="M6" s="10"/>
-      <c r="N6" s="10"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="10"/>
-      <c r="Q6" s="10"/>
-      <c r="R6" s="10"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="10"/>
-      <c r="U6" s="10"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="10"/>
-      <c r="X6" s="10"/>
-      <c r="Y6" s="10"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C7" s="2">
@@ -1146,7 +1128,7 @@
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="2">
@@ -1166,7 +1148,7 @@
       <c r="A9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="2">
@@ -1183,48 +1165,30 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="3">
         <v>17.008369</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="3">
         <v>-61.858765</v>
       </c>
-      <c r="E10" s="9">
+      <c r="E10" s="5">
         <v>46082.0</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="F10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="10"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="10"/>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="10"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="10"/>
-      <c r="U10" s="10"/>
-      <c r="V10" s="10"/>
-      <c r="W10" s="10"/>
-      <c r="X10" s="10"/>
-      <c r="Y10" s="10"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>17</v>
       </c>
       <c r="C11" s="8">
@@ -1237,7 +1201,7 @@
         <v>46082.0</v>
       </c>
       <c r="F11" s="10"/>
-      <c r="G11" s="6" t="s">
+      <c r="G11" s="7" t="s">
         <v>28</v>
       </c>
       <c r="H11" s="10"/>

</xml_diff>